<commit_message>
fix: make import template dropdowns Excel-compatible
</commit_message>
<xml_diff>
--- a/assets/templates/sisip-template-import.xlsx
+++ b/assets/templates/sisip-template-import.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panduan" sheetId="1" r:id="R58a33dd807be4654"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produk" sheetId="2" r:id="Rda8479204124490d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="3" r:id="R16dca76b5e4442c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referensi" sheetId="4" r:id="R00f7078ff8ca45b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panduan" sheetId="1" r:id="R994e08eceeae4237"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produk" sheetId="2" r:id="R05f38805faeb40cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="3" r:id="R604ad4e77c3e40df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referensi" sheetId="4" r:id="Rd964660645044fa1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1531,13 +1531,13 @@
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="E2:E201">
-      <x:formula1>'Referensi'!$B$2:$B$3</x:formula1>
+      <x:formula1>Pilihan SISIP,Populer</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="G2:I201">
-      <x:formula1>'Referensi'!$A$2:$A$11</x:formula1>
+      <x:formula1>Clean,Casual,Formal,Streetwear,Modest,Sporty,Vintage,Korean-inspired,Workwear,Party</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="J2:J201">
-      <x:formula1>'Referensi'!$C$2:$C$4</x:formula1>
+      <x:formula1>unisex,pria,wanita</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1737,13 +1737,13 @@
   </x:sheetData>
   <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="D2:D201">
-      <x:formula1>'Referensi'!$C$2:$C$4</x:formula1>
+      <x:formula1>unisex,pria,wanita</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F2:H201">
-      <x:formula1>'Referensi'!$A$2:$A$11</x:formula1>
+      <x:formula1>Clean,Casual,Formal,Streetwear,Modest,Sporty,Vintage,Korean-inspired,Workwear,Party</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I2:I201">
-      <x:formula1>'Referensi'!$D$2:$D$6</x:formula1>
+      <x:formula1>carbon,clay,mineral,olive,midnight</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="whole" operator="between" sqref="L2:L201">
       <x:formula1>1</x:formula1>

</xml_diff>

<commit_message>
feat: support general product websites
</commit_message>
<xml_diff>
--- a/assets/templates/sisip-template-import.xlsx
+++ b/assets/templates/sisip-template-import.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panduan" sheetId="1" r:id="R994e08eceeae4237"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produk" sheetId="2" r:id="R05f38805faeb40cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="3" r:id="R604ad4e77c3e40df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referensi" sheetId="4" r:id="Rd964660645044fa1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panduan" sheetId="1" r:id="R5f0d0237009d40d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produk" sheetId="2" r:id="R9f95a842625542df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Looks" sheetId="3" r:id="R897288349d52479b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referensi" sheetId="4" r:id="R5335307d09014b52"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -637,7 +637,7 @@
         <x:v>01</x:v>
       </x:c>
       <x:c r="B6" s="25" t="str">
-        <x:v>Isi dan import sheet Produk terlebih dahulu. Satu baris adalah satu warna; product_key yang sama akan menjadi satu produk dengan satu link Shopee.</x:v>
+        <x:v>Isi dan import sheet Produk terlebih dahulu. Satu baris adalah satu warna; product_key yang sama akan menjadi satu produk dengan satu link tujuan.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
@@ -671,7 +671,7 @@
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="47" t="str">
         <x:v>• URL gambar harus memakai https://.
-• Link affiliate wajib Shopee Indonesia.
+• Link tujuan wajib HTTPS. Shopee, TikTok Shop, dan website umum dikenali otomatis.
 • Hanya style SISIP pada dropdown yang diterima oleh import cepat.
 • Lihat sheet Referensi untuk seluruh pilihan valid.</x:v>
       </x:c>
@@ -874,7 +874,7 @@
         <x:v>Pleated Straight Trousers</x:v>
       </x:c>
       <x:c r="C4" s="68" t="str">
-        <x:v>https://shope.ee/contoh-link</x:v>
+        <x:v>https://shop.tiktok.com/view/product/contoh-link</x:v>
       </x:c>
       <x:c r="D4" s="71" t="n">
         <x:v>289000</x:v>
@@ -910,7 +910,7 @@
         <x:v>Leather Penny Loafers</x:v>
       </x:c>
       <x:c r="C5" s="69" t="str">
-        <x:v>https://shope.ee/contoh-link</x:v>
+        <x:v>https://brand.example.com/product/contoh</x:v>
       </x:c>
       <x:c r="D5" s="72" t="n">
         <x:v>319000</x:v>

</xml_diff>